<commit_message>
docs: record Option B curation scope
</commit_message>
<xml_diff>
--- a/docs/candidate_protein_curation.xlsx
+++ b/docs/candidate_protein_curation.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read This First" sheetId="1" r:id="Re1e88dffe06342d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate Proteins" sheetId="2" r:id="R4777673a8c044434"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read This First" sheetId="1" r:id="Read9414a82404583"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate Proteins" sheetId="2" r:id="R9b333c226431427d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -60,7 +60,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -87,6 +87,16 @@
         <x:fgColor rgb="FFFFF4D6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F0F3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F0F3"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -100,7 +110,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -152,6 +162,12 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -380,68 +396,68 @@
         <x:v>Read before assigning any training labels</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="48" customHeight="1">
-      <x:c r="A5" s="10" t="str">
+    <x:row r="5" ht="58" customHeight="1">
+      <x:c r="A5" s="26" t="str">
         <x:v>Current state</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
         <x:v>All entries below are literature-supported candidates only. Final training-label cells are intentionally blank.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="48" customHeight="1">
-      <x:c r="A6" s="10" t="str">
-        <x:v>What a positive means</x:v>
+    <x:row r="6" ht="58" customHeight="1">
+      <x:c r="A6" s="26" t="str">
+        <x:v>Positive label (1)</x:v>
       </x:c>
       <x:c r="B6" s="13" t="str">
-        <x:v>A team-approved, source-defined association with ischemic stroke. Some records concern risk before stroke; others are measured after stroke or relate to outcomes. Decide whether those belong to one label before combining them.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="48" customHeight="1">
-      <x:c r="A7" s="10" t="str">
-        <x:v>What a candidate negative means</x:v>
+        <x:v>Under Option B, use a human primary study that reports a protein in relation to ischemic stroke: occurrence/risk before stroke, measurement in patients after stroke, or severity/outcome. Record which evidence type it is. Exclude animal-only and review-only papers; keep uncertain cases unlabeled for team review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="58" customHeight="1">
+      <x:c r="A7" s="26" t="str">
+        <x:v>How to label candidates</x:v>
       </x:c>
       <x:c r="B7" s="13" t="str">
-        <x:v>No qualifying association found in the agreed source and search scope. It is not a confirmed biological negative. Do not label a protein negative only because this workbook does not list it.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="48" customHeight="1">
-      <x:c r="A8" s="10" t="str">
-        <x:v>Recommended first decision</x:v>
+        <x:v>For label 1, record a human ischemic-stroke study, protein, evidence type, PMID/link, and the result. For label 0, use only a candidate-negative protein that has no qualifying record under the same documented search sources and date; cite the search record. This is not a confirmed biological negative. If evidence is uncertain, leave the label blank and exclude it from training.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="58" customHeight="1">
+      <x:c r="A8" s="26" t="str">
+        <x:v>Agreed scope: Option B</x:v>
       </x:c>
       <x:c r="B8" s="13" t="str">
-        <x:v>Choose one consistent target definition: (A) proteins associated with ischemic-stroke occurrence/risk, or (B) proteins reported in ischemic-stroke patients, including post-onset biomarkers. Avoid mixing the two without explicitly choosing B.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="48" customHeight="1">
-      <x:c r="A9" s="10" t="str">
-        <x:v>NCBI sequence retrieval</x:v>
+        <x:v>A protein is a positive candidate (label 1) if a qualifying human primary study reports it in relation to ischemic stroke. This includes pre-event risk studies and measurements after stroke, such as biomarkers or outcomes. Keep the evidence category in the row; do not describe association as causation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="58" customHeight="1">
+      <x:c r="A9" s="26" t="str">
+        <x:v>Where sequences come from</x:v>
       </x:c>
       <x:c r="B9" s="13" t="str">
-        <x:v>After review, copy approved rows into data/raw/curated_labels.csv using the repo template. Use the exact RefSeq accession, run scripts/prepare_ncbi_dataset.py, and verify the fetched record and accession.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="48" customHeight="1">
-      <x:c r="A10" s="10" t="str">
+        <x:v>NCBI Protein supplies the sequence, not the stroke label. Use the exact RefSeq accession from an accepted curation row. The repo script scripts/prepare_ncbi_dataset.py fetches the human sequence and exports CSV, Excel, and FASTA. Review the returned accession and organism.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="58" customHeight="1">
+      <x:c r="A10" s="26" t="str">
         <x:v>AlphaFold's role</x:v>
       </x:c>
       <x:c r="B10" s="13" t="str">
-        <x:v>Optional structure interpretation or feature exploration only. AlphaFold predicts a protein structure from sequence; it does not predict stroke association. pLDDT is structural confidence, not confidence in a stroke label.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="48" customHeight="1">
-      <x:c r="A11" s="10" t="str">
+        <x:v>Optional structure interpretation or feature exploration only. AlphaFold predicts protein structure from sequence; it does not predict stroke association. pLDDT is structural confidence, not confidence in a stroke label.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="58" customHeight="1">
+      <x:c r="A11" s="26" t="str">
         <x:v>Important limitation</x:v>
       </x:c>
       <x:c r="B11" s="13" t="str">
-        <x:v>This five-protein starter list is not a sufficient or balanced training dataset. These candidates are not yet approved labels, and no model should be trained on this sheet as-is.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="48" customHeight="1">
-      <x:c r="A12" s="10" t="str">
+        <x:v>This five-protein starter list is not a sufficient or balanced training dataset. Candidate positives are not approved labels, no candidate negatives are supplied, and no model should be trained on this sheet as-is.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="58" customHeight="1">
+      <x:c r="A12" s="26" t="str">
         <x:v>Curation status choices</x:v>
       </x:c>
       <x:c r="B12" s="13" t="str">
-        <x:v>Pending review | Accepted under agreed rule | Rejected | Need more evidence</x:v>
+        <x:v>Pending review | Accepted under Option B | Rejected | Need more evidence</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>